<commit_message>
skript das alle vorhersagen in excel speichert
</commit_message>
<xml_diff>
--- a/output/predictions.xlsx
+++ b/output/predictions.xlsx
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.6845867017690147</v>
+        <v>0.6845896486801267</v>
       </c>
     </row>
     <row r="3">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.3383810410751992</v>
+        <v>0.3383857972536792</v>
       </c>
     </row>
     <row r="4">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.8041420785156048</v>
+        <v>0.804145446325978</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.8979115381258913</v>
+        <v>0.897913856430492</v>
       </c>
     </row>
     <row r="6">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.7569120894492523</v>
+        <v>0.7569124882504117</v>
       </c>
     </row>
     <row r="7">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.7451866231822964</v>
+        <v>0.7451915014857194</v>
       </c>
     </row>
     <row r="8">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.7607798726191958</v>
+        <v>0.7607836960144646</v>
       </c>
     </row>
     <row r="9">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.5903726450443131</v>
+        <v>0.5903595893520683</v>
       </c>
     </row>
     <row r="10">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.6994580825903529</v>
+        <v>0.6994563835279511</v>
       </c>
     </row>
   </sheetData>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5589844983313628</v>
+        <v>0.5589872319235494</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -753,25 +753,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Utah Jazz</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.4852912040259699</v>
+        <v>0.710714006852612</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
     </row>
@@ -783,25 +783,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.7107161905086252</v>
+        <v>0.4361005220957239</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.4626482946568332</v>
+        <v>0.4626511856295711</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -843,25 +843,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.4361035895025651</v>
+        <v>0.4852893920007732</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>New York Knicks</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6986761338295182</v>
+        <v>0.6986759429842281</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
boxscores angepasst -> 17.03 ACC von 100%
</commit_message>
<xml_diff>
--- a/output/predictions.xlsx
+++ b/output/predictions.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.7046881318092346</v>
+        <v>0.7294707894325256</v>
       </c>
       <c r="F2" t="n">
         <v>22500999</v>
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.3010091483592987</v>
+        <v>0.2842900454998016</v>
       </c>
       <c r="F3" t="n">
         <v>22501000</v>
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.2131834179162979</v>
+        <v>0.2439689189195633</v>
       </c>
       <c r="F4" t="n">
         <v>22501001</v>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.6208163499832153</v>
+        <v>0.5209299325942993</v>
       </c>
       <c r="F5" t="n">
         <v>22501002</v>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.6639977693557739</v>
+        <v>0.6554064154624939</v>
       </c>
       <c r="F6" t="n">
         <v>22501004</v>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6190536022186279</v>
+        <v>0.5324534177780151</v>
       </c>
       <c r="F7" t="n">
         <v>22501005</v>
@@ -635,11 +635,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.5686780214309692</v>
+        <v>0.494267612695694</v>
       </c>
       <c r="F8" t="n">
         <v>22500651</v>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.1298697739839554</v>
+        <v>0.1570685207843781</v>
       </c>
       <c r="F9" t="n">
         <v>22501006</v>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.3476361036300659</v>
+        <v>0.3276689648628235</v>
       </c>
       <c r="F10" t="n">
         <v>22501007</v>
@@ -760,29 +760,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.4343498349189758</v>
+        <v>0.2662922739982605</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>22500996</v>
+        <v>22500995</v>
       </c>
     </row>
     <row r="3">
@@ -793,29 +793,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Milwaukee Bucks</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.3743271231651306</v>
+        <v>0.5137976408004761</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>22500995</v>
+        <v>22500996</v>
       </c>
     </row>
     <row r="4">
@@ -826,29 +826,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Oklahoma City Thunder</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Oklahoma City Thunder</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.2116377651691437</v>
+        <v>0.3884319663047791</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Oklahoma City Thunder</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>22500992</v>
+        <v>22500998</v>
       </c>
     </row>
     <row r="5">
@@ -859,29 +859,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Indiana Pacers</t>
+          <t>Oklahoma City Thunder</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Oklahoma City Thunder</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.7550305724143982</v>
+        <v>0.2785426378250122</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Oklahoma City Thunder</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>22500994</v>
+        <v>22500992</v>
       </c>
     </row>
     <row r="6">
@@ -892,29 +892,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Miami Heat</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.5457360744476318</v>
+        <v>0.1558626741170883</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>22500991</v>
+        <v>22500993</v>
       </c>
     </row>
     <row r="7">
@@ -925,29 +925,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Washington Wizards</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.1621145457029343</v>
+        <v>0.5540216565132141</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>22500993</v>
+        <v>22500991</v>
       </c>
     </row>
     <row r="8">
@@ -958,29 +958,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.3026701211929321</v>
+        <v>0.8187637329101562</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>22500998</v>
+        <v>22500994</v>
       </c>
     </row>
     <row r="9">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.6574461460113525</v>
+        <v>0.6405219435691833</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
playoff schedule implemented and new features added
</commit_message>
<xml_diff>
--- a/output/predictions.xlsx
+++ b/output/predictions.xlsx
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.6051424145698547</v>
+        <v>0.6133015155792236</v>
       </c>
       <c r="F2" t="n">
         <v>42520001</v>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.5977880358695984</v>
+        <v>0.584772527217865</v>
       </c>
       <c r="F3" t="n">
         <v>42520007</v>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.7210045456886292</v>
+        <v>0.6660698056221008</v>
       </c>
       <c r="F4" t="n">
         <v>42520013</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.5657499432563782</v>
+        <v>0.5945318937301636</v>
       </c>
       <c r="F5" t="n">
         <v>42520031</v>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.7124065160751343</v>
+        <v>0.7690243721008301</v>
       </c>
       <c r="F6" t="n">
         <v>42520037</v>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6229561567306519</v>
+        <v>0.5765520930290222</v>
       </c>
       <c r="F7" t="n">
         <v>42520043</v>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.5598382949829102</v>
+        <v>0.5548051595687866</v>
       </c>
       <c r="F8" t="n">
         <v>42520019</v>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.7073587775230408</v>
+        <v>0.6796176433563232</v>
       </c>
       <c r="F9" t="n">
         <v>42520025</v>

</xml_diff>